<commit_message>
Faculty module enhancements and project updates
</commit_message>
<xml_diff>
--- a/Student_Import_Template.xlsx
+++ b/Student_Import_Template.xlsx
@@ -8,67 +8,125 @@
   </bookViews>
   <sheets>
     <sheet name="Students" sheetId="1" r:id="rId1"/>
+    <sheet name="Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Students!$A$1:$R$1</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="16">
-  <si>
-    <t>Student Name</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+  <si>
+    <t>* First Name</t>
+  </si>
+  <si>
+    <t>Middle Name</t>
+  </si>
+  <si>
+    <t>* Last Name</t>
+  </si>
+  <si>
+    <t>* Mobile Number</t>
+  </si>
+  <si>
+    <t>* Email Address</t>
   </si>
   <si>
     <t>PRN</t>
   </si>
   <si>
-    <t>Mobile</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Pramod bagade</t>
-  </si>
-  <si>
-    <t>pmb@gmail.com</t>
-  </si>
-  <si>
-    <t>student1</t>
-  </si>
-  <si>
-    <t>222222@gmail.com</t>
-  </si>
-  <si>
-    <t>student2</t>
-  </si>
-  <si>
-    <t>student3</t>
-  </si>
-  <si>
-    <t>student4</t>
-  </si>
-  <si>
-    <t>student5</t>
-  </si>
-  <si>
-    <t>student6</t>
-  </si>
-  <si>
-    <t>student7</t>
-  </si>
-  <si>
-    <t>student8</t>
-  </si>
-  <si>
-    <t>student9</t>
+    <t>Aadhaar Number</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Date of Birth</t>
+  </si>
+  <si>
+    <t>Parent Name</t>
+  </si>
+  <si>
+    <t>Parent Mobile</t>
+  </si>
+  <si>
+    <t>Parent Email</t>
+  </si>
+  <si>
+    <t>Permanent Address</t>
+  </si>
+  <si>
+    <t>Local Address</t>
+  </si>
+  <si>
+    <t>Emergency Contact Name</t>
+  </si>
+  <si>
+    <t>Emergency Contact Number</t>
+  </si>
+  <si>
+    <t>ABC ID</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>FacultyERP Student Import Instructions</t>
+  </si>
+  <si>
+    <t>1. Fields prefixed with * are mandatory.</t>
+  </si>
+  <si>
+    <t>2. Mobile Number must be unique.</t>
+  </si>
+  <si>
+    <t>3. Email Address must be unique.</t>
+  </si>
+  <si>
+    <t>4. PRN is optional during admission and can be updated later.</t>
+  </si>
+  <si>
+    <t>5. Aadhaar Number is optional.</t>
+  </si>
+  <si>
+    <t>6. Department, Course, Semester, Division and Academic Year are taken from the Student Master screen.</t>
+  </si>
+  <si>
+    <t>7. Do not modify the column headers.</t>
+  </si>
+  <si>
+    <t>Amit</t>
+  </si>
+  <si>
+    <t>Patil</t>
+  </si>
+  <si>
+    <t>Sneha</t>
+  </si>
+  <si>
+    <t>Joshi</t>
+  </si>
+  <si>
+    <t>sneha@test.com</t>
+  </si>
+  <si>
+    <t>amit@test.com</t>
+  </si>
+  <si>
+    <t>PRN1001</t>
+  </si>
+  <si>
+    <t>PRN1002</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -79,6 +137,12 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -90,15 +154,20 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -106,15 +175,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -415,13 +502,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:R6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="30" customWidth="1"/>
+    <col min="1" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="25" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="13" max="14" width="40" customWidth="1"/>
+    <col min="15" max="15" width="25" customWidth="1"/>
+    <col min="16" max="17" width="22" customWidth="1"/>
+    <col min="18" max="18" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -434,160 +534,151 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2">
-        <v>111111</v>
-      </c>
-      <c r="C2">
-        <v>1111111111</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2">
+        <v>9876543210</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3">
-        <v>222222</v>
-      </c>
-      <c r="C3">
-        <v>2222222222</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3">
+        <v>9876543211</v>
+      </c>
+      <c r="E3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="E4" s="3"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="E5" s="3"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="E6" s="3"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:R1"/>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="120" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4">
-        <v>222222</v>
-      </c>
-      <c r="C4">
-        <v>2222222222</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5">
-        <v>222222</v>
-      </c>
-      <c r="C5">
-        <v>2222222222</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6">
-        <v>222222</v>
-      </c>
-      <c r="C6">
-        <v>2222222222</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7">
-        <v>222222</v>
-      </c>
-      <c r="C7">
-        <v>2222222222</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8">
-        <v>222222</v>
-      </c>
-      <c r="C8">
-        <v>2222222222</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9">
-        <v>222222</v>
-      </c>
-      <c r="C9">
-        <v>2222222222</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10">
-        <v>222222</v>
-      </c>
-      <c r="C10">
-        <v>2222222222</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11">
-        <v>222222</v>
-      </c>
-      <c r="C11">
-        <v>2222222222</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1"/>
-    <hyperlink ref="D3" r:id="rId2"/>
-    <hyperlink ref="D4" r:id="rId3"/>
-    <hyperlink ref="D5" r:id="rId4"/>
-    <hyperlink ref="D6" r:id="rId5"/>
-    <hyperlink ref="D7" r:id="rId6"/>
-    <hyperlink ref="D8" r:id="rId7"/>
-    <hyperlink ref="D9" r:id="rId8"/>
-    <hyperlink ref="D10" r:id="rId9"/>
-    <hyperlink ref="D11" r:id="rId10"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>